<commit_message>
April 14 2025  Legal Matters changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1513_ClientGiftPre_ApprovalPage_AddingaRecipientToTheSelectedRecipientSection.xlsx
+++ b/TestData/LV_T1513_ClientGiftPre_ApprovalPage_AddingaRecipientToTheSelectedRecipientSection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3A9E9A9-9FC3-44F4-991D-64BFA2B74D88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075083CB-9FEC-4DC8-8779-D65AEE84D74F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -836,14 +836,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
@@ -851,7 +851,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -859,81 +859,81 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>56</v>
       </c>

</xml_diff>